<commit_message>
Update Playwright MCP defect reporting and project changes
</commit_message>
<xml_diff>
--- a/reports/Defects.xlsx
+++ b/reports/Defects.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AutomationProjects\qa-assignment\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FC123A0-4545-4BE8-BC6C-B4339B666702}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D0A59EC-1599-418F-967B-6AA22E2A3122}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{6B920BA3-4B0E-4699-BFAF-DCD173DE5E6B}"/>
   </bookViews>
@@ -60,31 +60,31 @@
     <t>DEF-001</t>
   </si>
   <si>
+    <t>Major</t>
+  </si>
+  <si>
+    <t>screenshots/login-failure.png</t>
+  </si>
+  <si>
     <t>Login</t>
   </si>
   <si>
-    <t>Failed Login failed</t>
-  </si>
-  <si>
-    <t>Open app → Enter invalid user</t>
-  </si>
-  <si>
-    <t>Error message displayed</t>
-  </si>
-  <si>
-    <t>Assertion failed</t>
-  </si>
-  <si>
-    <t>Major</t>
+    <t>Login failed with valid credentials</t>
+  </si>
+  <si>
+    <t>1. Open SauceDemo 2. Enter valid username/password 3. Click Login</t>
+  </si>
+  <si>
+    <t>User should navigate to inventory page</t>
+  </si>
+  <si>
+    <t>Login button failed due to timeout</t>
   </si>
   <si>
     <t>High</t>
   </si>
   <si>
     <t>Open</t>
-  </si>
-  <si>
-    <t>login-failed</t>
   </si>
 </sst>
 </file>
@@ -483,31 +483,31 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" t="s">
+      <c r="H2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" t="s">
         <v>12</v>
-      </c>
-      <c r="D2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J2" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>